<commit_message>
Mide que falta para jubilar las secciones 1-5
Agrega la hoja N4 al libro de validacion. Calcula, palabra por palabra,
cuales de las 36 formas que la app ya enseña NO se pueden pasar al modelo
nuevo, y por que.

El cuello de botella no es el esfuerzo: es la materia prima. De las 248
frases atestiguadas del corpus solo 110 son conversacionales; las otras
138 son descripciones en tercera persona ("El canasto grande") que no
pueden ser un turno de dialogo. Diecisiete palabras se quedaron sin una
sola frase usable, entre ellas las mas basicas: Eje, Takwa, Kuchi, Yawi,
Paki, Metzti y todos los terminos de parentesco.

La hoja trae una columna vacia por palabra. Una frase corta y natural
desbloquea cada una: convierte "validar todo el contenido" en un pedido
acotado que un hablante puede contestar en una sesion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/validacion-lecciones-artesanales.xlsx
+++ b/docs/validacion-lecciones-artesanales.xlsx
@@ -6,12 +6,13 @@
     <sheet name="N1. Diálogos (módulo nuevo)" sheetId="2" r:id="rId2"/>
     <sheet name="N2. Vocabulario (módulo nuevo)" sheetId="3" r:id="rId3"/>
     <sheet name="N3. Notas, tareas y preguntas" sheetId="4" r:id="rId4"/>
-    <sheet name="1. Vocabulario" sheetId="5" r:id="rId5"/>
-    <sheet name="2. Frases" sheetId="6" r:id="rId6"/>
-    <sheet name="3. Ejercicios" sheetId="7" r:id="rId7"/>
-    <sheet name="4. Cómo arma los ejercicios" sheetId="8" r:id="rId8"/>
-    <sheet name="5. Corpus" sheetId="9" r:id="rId9"/>
-    <sheet name="6. Preguntas" sheetId="10" r:id="rId10"/>
+    <sheet name="N4. Lo que falta" sheetId="5" r:id="rId5"/>
+    <sheet name="1. Vocabulario" sheetId="6" r:id="rId6"/>
+    <sheet name="2. Frases" sheetId="7" r:id="rId7"/>
+    <sheet name="3. Ejercicios" sheetId="8" r:id="rId8"/>
+    <sheet name="4. Cómo arma los ejercicios" sheetId="9" r:id="rId9"/>
+    <sheet name="5. Corpus" sheetId="10" r:id="rId10"/>
+    <sheet name="6. Preguntas" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -270,125 +271,137 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N4. Lo que falta</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LA HOJA MÁS ÚTIL SI HAY POCO TIEMPO. Las palabras que la app ya enseña pero que no se pueden pasar al modelo nuevo porque no existe ninguna frase donde se usen en conversación. Una frase corta por palabra desbloquea cada una.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">El contenido que ya está publicado (hojas 1 a 6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Vocabulario</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Las 36 palabras y expresiones que la app enseña hoy, con la página del diccionario donde se verificó cada una.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. Frases</t>
+          <t xml:space="preserve">1. Vocabulario</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Las 34 frases completas que aparecen en pantalla. Se distingue entre las copiadas de una fuente y las ARMADAS para un ejercicio: estas últimas son las que más riesgo tienen.</t>
+          <t xml:space="preserve">Las 36 palabras y expresiones que la app enseña hoy, con la página del diccionario donde se verificó cada una.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Ejercicios</t>
+          <t xml:space="preserve">2. Frases</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Los 178 ejercicios tal como los ve el estudiante, con su respuesta correcta y sus opciones falsas.</t>
+          <t xml:space="preserve">Las 34 frases completas que aparecen en pantalla. Se distingue entre las copiadas de una fuente y las ARMADAS para un ejercicio: estas últimas son las que más riesgo tienen.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Cómo arma los ejercicios</t>
+          <t xml:space="preserve">3. Ejercicios</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La app no guarda los ejercicios ya hechos: los arma en el momento. Aquí se explica qué decide la máquina y qué no, y se listan los pares de palabras que podrían confundirse.</t>
+          <t xml:space="preserve">Los 178 ejercicios tal como los ve el estudiante, con su respuesta correcta y sus opciones falsas.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. Corpus</t>
+          <t xml:space="preserve">4. Cómo arma los ejercicios</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qué se extrajo del diccionario, cuánto es, y una tabla para estimar qué costaría revisarlo.</t>
+          <t xml:space="preserve">La app no guarda los ejercicios ya hechos: los arma en el momento. Aquí se explica qué decide la máquina y qué no, y se listan los pares de palabras que podrían confundirse.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">5. Corpus</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué se extrajo del diccionario, cuánto es, y una tabla para estimar qué costaría revisarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">6. Preguntas</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Las preguntas concretas que quedaron abiertas.</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Sobre la columna "Evidencia"</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Directa</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La forma aparece tal cual en una fuente, con su página.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivada</t>
+          <t xml:space="preserve">Directa</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La forma se construyó aplicando una regla (por ejemplo, ponerle el prefijo "nu-" a una raíz). La regla está atestiguada; esa forma exacta no se encontró escrita. Son las que más necesitan confirmación.</t>
+          <t xml:space="preserve">La forma aparece tal cual en una fuente, con su página.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Derivada</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La forma se construyó aplicando una regla (por ejemplo, ponerle el prefijo "nu-" a una raíz). La regla está atestiguada; esa forma exacta no se encontró escrita. Son las que más necesitan confirmación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Sin localizar</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">No se pudo rastrear. Se enseña igual porque venía del material de origen, pero está sin respaldo documentado.</t>
         </is>
@@ -400,6 +413,384 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="66" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El corpus extraído del diccionario</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Es una base de datos armada a partir del YULTAJTAKETZALIS. De ella salen las lecciones generadas automáticamente, que hoy están APAGADAS en la app porque nadie las ha revisado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué contiene</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuánto</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Palabras</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <v>1012</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada una con su traducción, categoría gramatical, tema y la página de donde salió.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frases</t>
+        </is>
+      </c>
+      <c r="C6" s="2">
+        <v>248</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oraciones de ejemplo, la mayoría del propio diccionario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descomposiciones morfológicas</t>
+        </is>
+      </c>
+      <c r="C7" s="2">
+        <v>805</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada frase partida en sus piezas (prefijos de sujeto, objeto, posesivos). Se hicieron POR ALINEACIÓN AUTOMÁTICA: son lo menos confiable de todo el corpus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formas marcadas con guion</t>
+        </is>
+      </c>
+      <c r="C8" s="2">
+        <v>297</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El diccionario las escribe con guion inicial (−Pia, −Tukay): no van sueltas, exigen prefijo. La app ya las excluye de las lecciones generadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Páginas del diccionario tocadas</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <v>181</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rango 25–256. NO cubre las pp.26–51 (la parte gramatical inicial), y por eso algunas palabras de las lecciones no se pueden rastrear ahí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Palabras por categoría</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuántas</t>
+        </is>
+      </c>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verbos</t>
+        </is>
+      </c>
+      <c r="C12" s="2">
+        <v>428</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sustantivos</t>
+        </is>
+      </c>
+      <c r="C13" s="2">
+        <v>408</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partículas</t>
+        </is>
+      </c>
+      <c r="C14" s="2">
+        <v>102</v>
+      </c>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adjetivos</t>
+        </is>
+      </c>
+      <c r="C15" s="2">
+        <v>67</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saludos</t>
+        </is>
+      </c>
+      <c r="C16" s="2">
+        <v>6</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Números</t>
+        </is>
+      </c>
+      <c r="C17" s="2">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Para estimar el costo de validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los bloques van del más útil y barato al más caro. La idea es poder empezar por uno solo, no por todo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bloque</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ítems</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qué habría que revisar</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Horas</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A · Lo que la app ya enseña</t>
+        </is>
+      </c>
+      <c r="C22" s="2">
+        <v>70</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las hojas 1 y 2 de este libro: ortografía, significado y naturalidad de las frases.</t>
+        </is>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B · Palabras del corpus (forma y significado)</t>
+        </is>
+      </c>
+      <c r="C23" s="2">
+        <v>1012</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¿Está bien escrita? ¿Significa eso? Sin ejemplos ni gramática.</t>
+        </is>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C · Solo las formas con guion</t>
+        </is>
+      </c>
+      <c r="C24" s="2">
+        <v>297</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmar cuáles exigen prefijo y con cuál se enseñan. Es el error que más se repitió en la app.</t>
+        </is>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D · Frases del corpus</t>
+        </is>
+      </c>
+      <c r="C25" s="2">
+        <v>248</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¿Se dicen así? ¿La traducción es fiel?</t>
+        </is>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E · Descomposiciones morfológicas</t>
+        </is>
+      </c>
+      <c r="C26" s="2">
+        <v>805</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lo más caro y lo más delicado: verificar el análisis morfológico automático.</t>
+        </is>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Honorario por hora</t>
+        </is>
+      </c>
+      <c r="C28" s="3"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">← a llenar en la reunión</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modalidad que le acomoda</t>
+        </is>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por hora / por ítem / por bloque cerrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuánto podría avanzar por semana</t>
+        </is>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2795,6 +3186,800 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las 17 palabras que bloquean el reemplazo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Para pasar una palabra al modelo nuevo hace falta una frase donde se use de verdad, en primera o segunda persona. El diccionario da muchas frases, pero casi todas son descripciones ("El canasto grande") que no sirven como turno de conversación. Estas se quedaron sin ninguna. Una frase corta y natural por palabra alcanza para desbloquearla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N°</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Náhuat</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Significado en la app</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sec.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frases en el corpus</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usables</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La única usable, si la hay</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNA FRASE NATURAL CON ESTA PALABRA</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traducción</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eje</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tesu</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tesu datka</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">De nada</t>
+        </is>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tesu ninemi yek</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No estoy bien</t>
+        </is>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nunan</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mi mamá</t>
+        </is>
+      </c>
+      <c r="D8" s="2">
+        <v>2</v>
+      </c>
+      <c r="E8" s="2">
+        <v>5</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nutatanoy</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mi abuelo</t>
+        </is>
+      </c>
+      <c r="D9" s="2">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nuteku</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mi papá</t>
+        </is>
+      </c>
+      <c r="D10" s="2">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2">
+        <v>5</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piltzín</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Niño / Niña</t>
+        </is>
+      </c>
+      <c r="D11" s="2">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2">
+        <v>2</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Siwat</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mujer</t>
+        </is>
+      </c>
+      <c r="D12" s="2">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takat</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hombre</t>
+        </is>
+      </c>
+      <c r="D13" s="2">
+        <v>2</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nikuni</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yo bebo</t>
+        </is>
+      </c>
+      <c r="D14" s="2">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takwa</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comer</t>
+        </is>
+      </c>
+      <c r="D15" s="2">
+        <v>3</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwawit</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Árbol / Leña</t>
+        </is>
+      </c>
+      <c r="D16" s="2">
+        <v>4</v>
+      </c>
+      <c r="E16" s="2">
+        <v>3</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metzti</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luna</t>
+        </is>
+      </c>
+      <c r="D17" s="2">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kuchi</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dormir</t>
+        </is>
+      </c>
+      <c r="D18" s="2">
+        <v>5</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paki</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reír / Estar feliz</t>
+        </is>
+      </c>
+      <c r="D19" s="2">
+        <v>5</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yawi</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ir</t>
+        </is>
+      </c>
+      <c r="D20" s="2">
+        <v>5</v>
+      </c>
+      <c r="E20" s="2">
+        <v>2</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Et</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frijol</t>
+        </is>
+      </c>
+      <c r="D21" s="2">
+        <v>3</v>
+      </c>
+      <c r="E21" s="2">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nikmana ne et = Yo cuezo los frijoles (cocino)</t>
+        </is>
+      </c>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nikpia</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yo tengo</t>
+        </is>
+      </c>
+      <c r="D22" s="2">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Naja nikpia se almun shiwit = Yo tengo</t>
+        </is>
+      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kal</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Casa</t>
+        </is>
+      </c>
+      <c r="D23" s="2">
+        <v>4</v>
+      </c>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Niktajkwilua se kal = Yo dibujo una casa</t>
+        </is>
+      </c>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mistun</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gato</t>
+        </is>
+      </c>
+      <c r="D24" s="2">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2">
+        <v>4</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Naja nikalaktia ne mistun = Yo entro al gato</t>
+        </is>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <v>22</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelu</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perro</t>
+        </is>
+      </c>
+      <c r="D25" s="2">
+        <v>4</v>
+      </c>
+      <c r="E25" s="2">
+        <v>9</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nikpashalua ne pelu = Yo paseo al perro</t>
+        </is>
+      </c>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2">
+        <v>23</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agua</t>
+        </is>
+      </c>
+      <c r="D26" s="2">
+        <v>3</v>
+      </c>
+      <c r="E26" s="2">
+        <v>5</v>
+      </c>
+      <c r="F26" s="2">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Naja nikumima at = Yo tiro agua (lejos)</t>
+        </is>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
@@ -4544,7 +5729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -5678,7 +6863,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -13050,7 +14235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -13319,382 +14504,4 @@
   </dataValidations>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="66" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El corpus extraído del diccionario</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Es una base de datos armada a partir del YULTAJTAKETZALIS. De ella salen las lecciones generadas automáticamente, que hoy están APAGADAS en la app porque nadie las ha revisado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qué contiene</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cuánto</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detalle</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Palabras</t>
-        </is>
-      </c>
-      <c r="C5" s="2">
-        <v>1012</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cada una con su traducción, categoría gramatical, tema y la página de donde salió.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Frases</t>
-        </is>
-      </c>
-      <c r="C6" s="2">
-        <v>248</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Oraciones de ejemplo, la mayoría del propio diccionario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Descomposiciones morfológicas</t>
-        </is>
-      </c>
-      <c r="C7" s="2">
-        <v>805</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cada frase partida en sus piezas (prefijos de sujeto, objeto, posesivos). Se hicieron POR ALINEACIÓN AUTOMÁTICA: son lo menos confiable de todo el corpus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Formas marcadas con guion</t>
-        </is>
-      </c>
-      <c r="C8" s="2">
-        <v>297</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El diccionario las escribe con guion inicial (−Pia, −Tukay): no van sueltas, exigen prefijo. La app ya las excluye de las lecciones generadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Páginas del diccionario tocadas</t>
-        </is>
-      </c>
-      <c r="C9" s="2">
-        <v>181</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rango 25–256. NO cubre las pp.26–51 (la parte gramatical inicial), y por eso algunas palabras de las lecciones no se pueden rastrear ahí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Palabras por categoría</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cuántas</t>
-        </is>
-      </c>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Verbos</t>
-        </is>
-      </c>
-      <c r="C12" s="2">
-        <v>428</v>
-      </c>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sustantivos</t>
-        </is>
-      </c>
-      <c r="C13" s="2">
-        <v>408</v>
-      </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partículas</t>
-        </is>
-      </c>
-      <c r="C14" s="2">
-        <v>102</v>
-      </c>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adjetivos</t>
-        </is>
-      </c>
-      <c r="C15" s="2">
-        <v>67</v>
-      </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saludos</t>
-        </is>
-      </c>
-      <c r="C16" s="2">
-        <v>6</v>
-      </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Números</t>
-        </is>
-      </c>
-      <c r="C17" s="2">
-        <v>1</v>
-      </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Para estimar el costo de validar</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Los bloques van del más útil y barato al más caro. La idea es poder empezar por uno solo, no por todo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bloque</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ítems</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qué habría que revisar</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Horas</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Costo</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comentario</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A · Lo que la app ya enseña</t>
-        </is>
-      </c>
-      <c r="C22" s="2">
-        <v>70</v>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Las hojas 1 y 2 de este libro: ortografía, significado y naturalidad de las frases.</t>
-        </is>
-      </c>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">B · Palabras del corpus (forma y significado)</t>
-        </is>
-      </c>
-      <c r="C23" s="2">
-        <v>1012</v>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">¿Está bien escrita? ¿Significa eso? Sin ejemplos ni gramática.</t>
-        </is>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C · Solo las formas con guion</t>
-        </is>
-      </c>
-      <c r="C24" s="2">
-        <v>297</v>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmar cuáles exigen prefijo y con cuál se enseñan. Es el error que más se repitió en la app.</t>
-        </is>
-      </c>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">D · Frases del corpus</t>
-        </is>
-      </c>
-      <c r="C25" s="2">
-        <v>248</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">¿Se dicen así? ¿La traducción es fiel?</t>
-        </is>
-      </c>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E · Descomposiciones morfológicas</t>
-        </is>
-      </c>
-      <c r="C26" s="2">
-        <v>805</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lo más caro y lo más delicado: verificar el análisis morfológico automático.</t>
-        </is>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Honorario por hora</t>
-        </is>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">← a llenar en la reunión</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Modalidad que le acomoda</t>
-        </is>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">por hora / por ítem / por bloque cerrado</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cuánto podría avanzar por semana</t>
-        </is>
-      </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>